<commit_message>
New Functions file added
</commit_message>
<xml_diff>
--- a/Excel/Left,Right,Find_functions.xlsx
+++ b/Excel/Left,Right,Find_functions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Arbor all Folder\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E4A539-E75F-44FB-8313-9BD43D6EF059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1975CFA1-E613-411E-BEFB-F6474E8A8312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AD209C9D-020F-4DF3-B9C1-46D5CAA58059}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="74">
   <si>
     <t>Description</t>
   </si>
@@ -142,6 +142,120 @@
   </si>
   <si>
     <t>Vaishnavi Santosh Ubale</t>
+  </si>
+  <si>
+    <t>Sudarshan</t>
+  </si>
+  <si>
+    <t>Sujit</t>
+  </si>
+  <si>
+    <t>Raju</t>
+  </si>
+  <si>
+    <t>Abhishek</t>
+  </si>
+  <si>
+    <t>Arun</t>
+  </si>
+  <si>
+    <t>Ashok</t>
+  </si>
+  <si>
+    <t>Suraj</t>
+  </si>
+  <si>
+    <t>Sanjay</t>
+  </si>
+  <si>
+    <t>Asaram</t>
+  </si>
+  <si>
+    <t>Vilas</t>
+  </si>
+  <si>
+    <t>Abhijeet</t>
+  </si>
+  <si>
+    <t>Prashant</t>
+  </si>
+  <si>
+    <t>Uttam</t>
+  </si>
+  <si>
+    <t>Santosh</t>
+  </si>
+  <si>
+    <t>Wavhal</t>
+  </si>
+  <si>
+    <t>Kamble</t>
+  </si>
+  <si>
+    <t>Pardesi</t>
+  </si>
+  <si>
+    <t>Lohare</t>
+  </si>
+  <si>
+    <t>Dhavale</t>
+  </si>
+  <si>
+    <t>Jadhav</t>
+  </si>
+  <si>
+    <t>Rathod</t>
+  </si>
+  <si>
+    <t>Shelke</t>
+  </si>
+  <si>
+    <t>Bartakke</t>
+  </si>
+  <si>
+    <t>Thorve</t>
+  </si>
+  <si>
+    <t>Patil</t>
+  </si>
+  <si>
+    <t>Patle</t>
+  </si>
+  <si>
+    <t>Ubale</t>
+  </si>
+  <si>
+    <t>Sagar</t>
+  </si>
+  <si>
+    <t>Jitendra</t>
+  </si>
+  <si>
+    <t>Krushna</t>
+  </si>
+  <si>
+    <t>Amit</t>
+  </si>
+  <si>
+    <t>Dhanashree</t>
+  </si>
+  <si>
+    <t>Vaishnavi</t>
+  </si>
+  <si>
+    <t>Rushikesh</t>
+  </si>
+  <si>
+    <t>Ganesh</t>
+  </si>
+  <si>
+    <t>Omkar</t>
+  </si>
+  <si>
+    <t>Anjali</t>
+  </si>
+  <si>
+    <t>Mayank</t>
   </si>
 </sst>
 </file>
@@ -516,16 +630,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E55DF59E-995D-4DA0-941A-D4E6B0D04CAB}">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -539,7 +653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -555,16 +669,8 @@
         <f>RIGHT(A2,LEN(A2)-FIND(": ",A2))</f>
         <v xml:space="preserve"> 208011</v>
       </c>
-      <c r="G2">
-        <f>FIND(":",A2)</f>
-        <v>16</v>
-      </c>
-      <c r="I2">
-        <f>FIND("/",A2)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -577,11 +683,11 @@
         <v>Delhi</v>
       </c>
       <c r="D3" s="2" t="str">
-        <f t="shared" ref="D3:D15" si="2">RIGHT(A3,LEN(A3)-FIND(": ",A3))</f>
+        <f t="shared" ref="D3:D14" si="2">RIGHT(A3,LEN(A3)-FIND(": ",A3))</f>
         <v xml:space="preserve"> 208012</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -598,7 +704,7 @@
         <v xml:space="preserve"> 208013</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -615,7 +721,7 @@
         <v xml:space="preserve"> 208014</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -632,7 +738,7 @@
         <v xml:space="preserve"> 2080159</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -649,7 +755,7 @@
         <v xml:space="preserve"> 208016</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -666,7 +772,7 @@
         <v xml:space="preserve"> 208017</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
@@ -683,7 +789,7 @@
         <v xml:space="preserve"> 208018</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -700,7 +806,7 @@
         <v xml:space="preserve"> 208019</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
@@ -717,7 +823,7 @@
         <v xml:space="preserve"> 208020</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
@@ -734,7 +840,7 @@
         <v xml:space="preserve"> 208021</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
@@ -751,7 +857,7 @@
         <v xml:space="preserve"> 208022</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
@@ -768,7 +874,7 @@
         <v xml:space="preserve"> 208023</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -803,238 +909,196 @@
       <c r="A18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="2" t="str">
-        <f>LEFT(A18,FIND(" ",A18)-1)</f>
-        <v>Abhishek</v>
-      </c>
-      <c r="C18" s="2" t="str">
-        <f>MID(A18,FIND(" ",A18),FIND(" ",A18)+2)</f>
-        <v xml:space="preserve"> Sudarshan </v>
-      </c>
-      <c r="D18" s="2" t="str">
-        <f>RIGHT(A18,LEN(A18)-FIND(" ",A18))</f>
-        <v>Sudarshan Wavhal</v>
+      <c r="B18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="2" t="str">
-        <f t="shared" ref="B19:B31" si="3">LEFT(A19,FIND(" ",A19)-1)</f>
-        <v>Sagar</v>
-      </c>
-      <c r="C19" s="2" t="str">
-        <f>MID(A19,FIND(" ",A19),FIND(" ",A19)+2)</f>
-        <v xml:space="preserve"> Sujit K</v>
-      </c>
-      <c r="D19" s="2" t="str">
-        <f>RIGHT(A19,LEN(A19)-FIND(" ",A19))</f>
-        <v xml:space="preserve">Sujit Kamble </v>
+      <c r="B19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Jitendra</v>
-      </c>
-      <c r="C20" s="2" t="str">
-        <f t="shared" ref="C20:C31" si="4">MID(A20,FIND(" ",A20),FIND(" ",A20)+2)</f>
-        <v xml:space="preserve"> Raju Parde</v>
-      </c>
-      <c r="D20" s="2" t="str">
-        <f t="shared" ref="D19:D31" si="5">RIGHT(A20,FIND(" ",A20))</f>
-        <v>u Pardesi</v>
+      <c r="B20" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Krushna</v>
-      </c>
-      <c r="C21" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Abhishek </v>
-      </c>
-      <c r="D21" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>k Lohare</v>
+      <c r="B21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Amit</v>
-      </c>
-      <c r="C22" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Arun D</v>
-      </c>
-      <c r="D22" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>avale</v>
+      <c r="B22" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Dhanashree</v>
-      </c>
-      <c r="C23" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Ashok Jadhav</v>
-      </c>
-      <c r="D23" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>shok Jadhav</v>
+      <c r="B23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Vaishnavi</v>
-      </c>
-      <c r="C24" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Suraj Ratho</v>
-      </c>
-      <c r="D24" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>raj Rathod</v>
+      <c r="B24" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Suraj</v>
-      </c>
-      <c r="C25" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Sanjay </v>
-      </c>
-      <c r="D25" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>Shelke</v>
+      <c r="B25" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Rushikesh</v>
-      </c>
-      <c r="C26" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Asaram Bart</v>
-      </c>
-      <c r="D26" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>m Bartakke</v>
+      <c r="B26" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Ganesh</v>
-      </c>
-      <c r="C27" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Vilas Ja</v>
-      </c>
-      <c r="D27" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve"> Jadhav</v>
+      <c r="B27" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Omkar</v>
-      </c>
-      <c r="C28" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Abhijee</v>
-      </c>
-      <c r="D28" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>Thorve</v>
+      <c r="B28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Anjali</v>
-      </c>
-      <c r="C29" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Prashant</v>
-      </c>
-      <c r="D29" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>t Patil</v>
+      <c r="B29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Mayank</v>
-      </c>
-      <c r="C30" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Uttam Pa</v>
-      </c>
-      <c r="D30" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>m Patle</v>
+      <c r="B30" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Vaishnavi</v>
-      </c>
-      <c r="C31" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve"> Santosh Uba</v>
-      </c>
-      <c r="D31" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>tosh Ubale</v>
+      <c r="B31" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>